<commit_message>
feat: journaux d'encaissements consolidés, décalages de dates et exports enrichis
- Prise en charge du journal des encaissements consolidé du mois complet (01 au 30/31) avec détection des dates et ventilation automatique par jour
- Rapprochement avec tolérance de décalage de dates (date drift ±3 jours) et observations d'audit précises
- Export Excel coloré du rapprochement à 7 colonnes (Date, Client, Référence OM, Montant journal, Montant OM, Statut, Observation) avec surbrillances conditionnelles
- Option 'Toutes les journées' dans le sélecteur du rapprochement pour consultation et export mensuel consolidé
- Précision détaillée des opérations bloquantes dans la synthèse du rapport d'audit
- Migration complète du journal des arrhes vers le journal des encaissements avec couverture mensuelle robuste
- 185 tests unitaires et d'intégration validés
</commit_message>
<xml_diff>
--- a/tests/fixtures/releve_om_exemple.xlsx
+++ b/tests/fixtures/releve_om_exemple.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:Q36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1518,37 +1518,106 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" t="n">
+        <v>10</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>10:15:00</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>MP260520.1015.I00010</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Merchant Payment</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Succès</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>USSD</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>600000002</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>690000018</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="O35" t="n">
+        <v>45000</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>-450</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Relevé de vos opérations</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Transactions réussies</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Wallet Normal</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>600000002</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t>Solde final</t>
         </is>
       </c>
-      <c r="O35" t="n">
+      <c r="O36" t="n">
         <v>95000</v>
       </c>
     </row>

</xml_diff>